<commit_message>
Functionality of WorkBook with Performance Milestones & Planner
</commit_message>
<xml_diff>
--- a/data/Yes Prep Performance_Project Plan (Formulated).xlsx
+++ b/data/Yes Prep Performance_Project Plan (Formulated).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CSOD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A5ACAB-04F4-422B-A289-E23352EF0D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9CCB29-16A6-489A-B585-E07D2FC7AE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="153">
   <si>
     <t>S.No</t>
   </si>
@@ -288,9 +288,6 @@
     <t>Officially start the project with all stakeholders; review scope, roles, and timelines.</t>
   </si>
   <si>
-    <t>Rajesh</t>
-  </si>
-  <si>
     <t>Completed</t>
   </si>
   <si>
@@ -303,9 +300,6 @@
     <t>Ensure client has access to Cornerstone resources and training materials.</t>
   </si>
   <si>
-    <t>Yes Prep</t>
-  </si>
-  <si>
     <t>Customer will complete quiestionnaire and provide any document to help understand current processes and needs</t>
   </si>
   <si>
@@ -318,9 +312,6 @@
     <t>Discuss business needs and validate requirements for Performance setup.</t>
   </si>
   <si>
-    <t>Sharmila</t>
-  </si>
-  <si>
     <t>OU Work shop</t>
   </si>
   <si>
@@ -330,9 +321,6 @@
     <t>Align IT and integration teams on environment setup, SSO, and data migration.</t>
   </si>
   <si>
-    <t>Jeeva</t>
-  </si>
-  <si>
     <t>Set up recurring weekly project status meetings</t>
   </si>
   <si>
@@ -381,9 +369,6 @@
     <t>Conduct training sessions for client admins covering setup, workflows, performance cycles, reports, and troubleshooting.</t>
   </si>
   <si>
-    <t>Sharmila/Yes Prep</t>
-  </si>
-  <si>
     <t>Admin Training Session 2</t>
   </si>
   <si>
@@ -513,7 +498,7 @@
     <t>Customer</t>
   </si>
   <si>
-    <t>Customer + Business Consultant</t>
+    <t>Customer/Business Consultant</t>
   </si>
 </sst>
 </file>
@@ -2838,7 +2823,7 @@
     <col min="11" max="16384" width="8.77734375" style="33"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="45" t="s">
         <v>1</v>
       </c>
@@ -2869,11 +2854,8 @@
       <c r="J1" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="K1" s="33" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="44" t="s">
         <v>79</v>
       </c>
@@ -2891,7 +2873,7 @@
       </c>
       <c r="J2" s="49"/>
     </row>
-    <row r="3" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="35" t="s">
         <v>13</v>
       </c>
@@ -2906,22 +2888,19 @@
       <c r="F3" s="40"/>
       <c r="G3" s="40"/>
       <c r="H3" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="I3" s="41" t="s">
         <v>82</v>
       </c>
-      <c r="I3" s="41" t="s">
+      <c r="J3" s="41"/>
+    </row>
+    <row r="4" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="35" t="s">
         <v>83</v>
       </c>
-      <c r="J3" s="41"/>
-      <c r="K3" s="33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="35" t="s">
+      <c r="B4" s="52" t="s">
         <v>84</v>
-      </c>
-      <c r="B4" s="52" t="s">
-        <v>85</v>
       </c>
       <c r="C4" s="35">
         <v>0</v>
@@ -2931,22 +2910,19 @@
       <c r="F4" s="40"/>
       <c r="G4" s="40"/>
       <c r="H4" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="I4" s="41" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="41" t="s">
-        <v>83</v>
-      </c>
       <c r="J4" s="41"/>
-      <c r="K4" s="33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="35" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="52" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="35">
         <v>15</v>
@@ -2956,22 +2932,19 @@
       <c r="F5" s="40"/>
       <c r="G5" s="40"/>
       <c r="H5" s="41" t="s">
-        <v>87</v>
+        <v>151</v>
       </c>
       <c r="I5" s="41" t="s">
         <v>80</v>
       </c>
       <c r="J5" s="41"/>
-      <c r="K5" s="33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="50" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C6" s="35">
         <v>0</v>
@@ -2981,22 +2954,19 @@
       <c r="F6" s="40"/>
       <c r="G6" s="40"/>
       <c r="H6" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I6" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="41" t="s">
+      <c r="J6" s="41"/>
+    </row>
+    <row r="7" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="51" t="s">
         <v>89</v>
-      </c>
-      <c r="J6" s="41"/>
-      <c r="K6" s="33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>91</v>
       </c>
       <c r="C7" s="35">
         <v>0</v>
@@ -3006,22 +2976,19 @@
       <c r="F7" s="40"/>
       <c r="G7" s="40"/>
       <c r="H7" s="41" t="s">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="I7" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J7" s="41"/>
-      <c r="K7" s="33" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="35" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C8" s="35">
         <v>0</v>
@@ -3031,22 +2998,19 @@
       <c r="F8" s="40"/>
       <c r="G8" s="40"/>
       <c r="H8" s="41" t="s">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="I8" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J8" s="41"/>
-      <c r="K8" s="33" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
         <v>35</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C9" s="35">
         <v>0</v>
@@ -3056,22 +3020,19 @@
       <c r="F9" s="40"/>
       <c r="G9" s="40"/>
       <c r="H9" s="41" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="I9" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J9" s="41"/>
-      <c r="K9" s="33" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="35" t="s">
         <v>27</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C10" s="35">
         <v>0</v>
@@ -3081,22 +3042,19 @@
       <c r="F10" s="40"/>
       <c r="G10" s="40"/>
       <c r="H10" s="41" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
       <c r="I10" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J10" s="41"/>
-      <c r="K10" s="33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C11" s="35">
         <v>5</v>
@@ -3106,22 +3064,19 @@
       <c r="F11" s="40"/>
       <c r="G11" s="40"/>
       <c r="H11" s="41" t="s">
-        <v>82</v>
+        <v>134</v>
       </c>
       <c r="I11" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J11" s="41"/>
-      <c r="K11" s="33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="35" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C12" s="35">
         <v>2</v>
@@ -3131,22 +3086,19 @@
       <c r="F12" s="40"/>
       <c r="G12" s="40"/>
       <c r="H12" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I12" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I12" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J12" s="41"/>
-      <c r="K12" s="33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="35" t="s">
         <v>60</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C13" s="35">
         <v>2</v>
@@ -3156,22 +3108,19 @@
       <c r="F13" s="40"/>
       <c r="G13" s="40"/>
       <c r="H13" s="41" t="s">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="I13" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J13" s="41"/>
-      <c r="K13" s="33" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="35" t="s">
         <v>61</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C14" s="35">
         <v>0</v>
@@ -3181,22 +3130,19 @@
       <c r="F14" s="40"/>
       <c r="G14" s="40"/>
       <c r="H14" s="41" t="s">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="I14" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J14" s="43"/>
-      <c r="K14" s="33" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="35" t="s">
         <v>46</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C15" s="35">
         <f>E15-D15</f>
@@ -3207,22 +3153,19 @@
       <c r="F15" s="40"/>
       <c r="G15" s="40"/>
       <c r="H15" s="41" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="I15" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J15" s="41"/>
-      <c r="K15" s="33" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="35" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B16" s="52" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C16" s="35">
         <v>2</v>
@@ -3232,22 +3175,19 @@
       <c r="F16" s="40"/>
       <c r="G16" s="40"/>
       <c r="H16" s="41" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="I16" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J16" s="41"/>
-      <c r="K16" s="33" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="17" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="35" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B17" s="52" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C17" s="35">
         <v>2</v>
@@ -3257,22 +3197,19 @@
       <c r="F17" s="40"/>
       <c r="G17" s="40"/>
       <c r="H17" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I17" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J17" s="41"/>
-      <c r="K17" s="33" t="s">
-        <v>156</v>
-      </c>
     </row>
     <row r="18" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="35" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C18" s="35">
         <v>2</v>
@@ -3282,22 +3219,19 @@
       <c r="F18" s="40"/>
       <c r="G18" s="40"/>
       <c r="H18" s="41" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="I18" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J18" s="41"/>
-      <c r="K18" s="33" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="19" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="35" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B19" s="35" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C19" s="35">
         <v>3</v>
@@ -3307,22 +3241,19 @@
       <c r="F19" s="40"/>
       <c r="G19" s="40"/>
       <c r="H19" s="41" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="I19" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J19" s="41"/>
-      <c r="K19" s="33" t="s">
-        <v>157</v>
-      </c>
     </row>
     <row r="20" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="35" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C20" s="35">
         <v>0</v>
@@ -3332,22 +3263,19 @@
       <c r="F20" s="40"/>
       <c r="G20" s="40"/>
       <c r="H20" s="41" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="I20" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J20" s="41"/>
-      <c r="K20" s="33" t="s">
-        <v>157</v>
-      </c>
     </row>
     <row r="21" spans="1:11" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="35" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C21" s="35">
         <v>0</v>
@@ -3357,22 +3285,19 @@
       <c r="F21" s="40"/>
       <c r="G21" s="40"/>
       <c r="H21" s="41" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="I21" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J21" s="41"/>
-      <c r="K21" s="33" t="s">
-        <v>157</v>
-      </c>
     </row>
     <row r="22" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="35" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C22" s="35">
         <v>0</v>
@@ -3382,22 +3307,19 @@
       <c r="F22" s="40"/>
       <c r="G22" s="40"/>
       <c r="H22" s="41" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="I22" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J22" s="41"/>
-      <c r="K22" s="33" t="s">
-        <v>157</v>
-      </c>
     </row>
     <row r="23" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="35" t="s">
         <v>34</v>
       </c>
       <c r="B23" s="52" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C23" s="35">
         <v>0</v>
@@ -3407,22 +3329,19 @@
       <c r="F23" s="40"/>
       <c r="G23" s="40"/>
       <c r="H23" s="41" t="s">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="I23" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J23" s="41"/>
-      <c r="K23" s="33" t="s">
-        <v>137</v>
-      </c>
     </row>
     <row r="24" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="35" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C24" s="35">
         <v>0</v>
@@ -3432,22 +3351,19 @@
       <c r="F24" s="40"/>
       <c r="G24" s="40"/>
       <c r="H24" s="41" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="I24" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J24" s="41"/>
-      <c r="K24" s="33" t="s">
-        <v>157</v>
-      </c>
     </row>
     <row r="25" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="35" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B25" s="52" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C25" s="35">
         <v>0</v>
@@ -3457,22 +3373,19 @@
       <c r="F25" s="40"/>
       <c r="G25" s="40"/>
       <c r="H25" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I25" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I25" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J25" s="41"/>
-      <c r="K25" s="33" t="s">
-        <v>156</v>
-      </c>
     </row>
     <row r="26" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B26" s="52" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C26" s="35">
         <v>0</v>
@@ -3482,22 +3395,19 @@
       <c r="F26" s="40"/>
       <c r="G26" s="40"/>
       <c r="H26" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I26" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I26" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J26" s="41"/>
-      <c r="K26" s="33" t="s">
-        <v>156</v>
-      </c>
     </row>
     <row r="27" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="35" t="s">
         <v>71</v>
       </c>
       <c r="B27" s="52" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C27" s="35">
         <v>0</v>
@@ -3507,22 +3417,19 @@
       <c r="F27" s="40"/>
       <c r="G27" s="40"/>
       <c r="H27" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I27" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I27" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J27" s="41"/>
-      <c r="K27" s="33" t="s">
-        <v>156</v>
-      </c>
     </row>
     <row r="28" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="35" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B28" s="52" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C28" s="35">
         <v>2</v>
@@ -3532,22 +3439,19 @@
       <c r="F28" s="40"/>
       <c r="G28" s="40"/>
       <c r="H28" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I28" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I28" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J28" s="41"/>
-      <c r="K28" s="33" t="s">
-        <v>156</v>
-      </c>
     </row>
     <row r="29" spans="1:11" s="34" customFormat="1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="35" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B29" s="52" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C29" s="35">
         <v>5</v>
@@ -3557,22 +3461,20 @@
       <c r="F29" s="40"/>
       <c r="G29" s="54"/>
       <c r="H29" s="41" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="I29" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J29" s="41"/>
-      <c r="K29" s="33" t="s">
-        <v>142</v>
-      </c>
+      <c r="K29" s="33"/>
     </row>
     <row r="30" spans="1:11" s="34" customFormat="1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="35" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B30" s="52" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C30" s="35">
         <v>2</v>
@@ -3582,22 +3484,20 @@
       <c r="F30" s="40"/>
       <c r="G30" s="42"/>
       <c r="H30" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I30" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I30" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J30" s="41"/>
-      <c r="K30" s="33" t="s">
-        <v>156</v>
-      </c>
+      <c r="K30" s="33"/>
     </row>
     <row r="31" spans="1:11" s="34" customFormat="1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="35" t="s">
         <v>63</v>
       </c>
       <c r="B31" s="52" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C31" s="35">
         <v>3</v>
@@ -3607,22 +3507,20 @@
       <c r="F31" s="40"/>
       <c r="G31" s="42"/>
       <c r="H31" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I31" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I31" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J31" s="41"/>
-      <c r="K31" s="33" t="s">
-        <v>156</v>
-      </c>
+      <c r="K31" s="33"/>
     </row>
     <row r="32" spans="1:11" s="34" customFormat="1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="35" t="s">
         <v>75</v>
       </c>
       <c r="B32" s="52" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C32" s="35">
         <v>2</v>
@@ -3632,22 +3530,20 @@
       <c r="F32" s="40"/>
       <c r="G32" s="42"/>
       <c r="H32" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I32" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I32" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J32" s="41"/>
-      <c r="K32" s="33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K32" s="33"/>
+    </row>
+    <row r="33" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="43" t="s">
         <v>76</v>
       </c>
       <c r="B33" s="52" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C33" s="43">
         <v>2</v>
@@ -3657,15 +3553,12 @@
       <c r="F33" s="41"/>
       <c r="G33" s="41"/>
       <c r="H33" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="I33" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="I33" s="41" t="s">
-        <v>89</v>
-      </c>
       <c r="J33" s="41"/>
-      <c r="K33" s="33" t="s">
-        <v>156</v>
-      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J33" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -3697,41 +3590,41 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C5" s="24"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C7" s="24"/>
     </row>
@@ -3751,93 +3644,93 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C12" s="24"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C13" s="24"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="37" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C14" s="24"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="37" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C15" s="24"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="37" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C16" s="24"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="37" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C17" s="24"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="37" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C18" s="24"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="37" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B19" s="35" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C19" s="24"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="37" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C20" s="24"/>
     </row>
@@ -3864,12 +3757,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cb26c466-b7e7-420d-9d7a-8be07dface07" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Notes xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
+    <Type_x002f_DataAlignment xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Portal xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
+    <Location xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
+    <Seismic_x0020_Tag xmlns="cb26c466-b7e7-420d-9d7a-8be07dface07">External</Seismic_x0020_Tag>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4231,27 +4133,28 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cb26c466-b7e7-420d-9d7a-8be07dface07" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Notes xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
-    <Type_x002f_DataAlignment xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Portal xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
-    <Location xmlns="97137d12-c5e7-4bf8-ab63-816b90ba6850" xsi:nil="true"/>
-    <Seismic_x0020_Tag xmlns="cb26c466-b7e7-420d-9d7a-8be07dface07">External</Seismic_x0020_Tag>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9E18508-EFC6-4E64-8939-60B8F0DCA946}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFE8543E-662C-4B0C-8B28-0C97DF0FB3AC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="cb26c466-b7e7-420d-9d7a-8be07dface07"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="97137d12-c5e7-4bf8-ab63-816b90ba6850"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4277,19 +4180,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFE8543E-662C-4B0C-8B28-0C97DF0FB3AC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9E18508-EFC6-4E64-8939-60B8F0DCA946}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="cb26c466-b7e7-420d-9d7a-8be07dface07"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="97137d12-c5e7-4bf8-ab63-816b90ba6850"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>